<commit_message>
fix(var-menu-001): repair recalculation and date validation
</commit_message>
<xml_diff>
--- a/docs/07-operations/var-menu-001/VKM-001_MARGHERITA_CHEF_MANAGER_APPROVAL_DRAFT_v1.0.0.xlsx
+++ b/docs/07-operations/var-menu-001/VKM-001_MARGHERITA_CHEF_MANAGER_APPROVAL_DRAFT_v1.0.0.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="КАЛЬКУЛЯЦИЯ" sheetId="1" r:id="R4b0a3aceeb304b53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ТЕХКАРТА" sheetId="2" r:id="R26b192f3cdc94062"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="АНКЕТА" sheetId="3" r:id="R53254e2e9da74d6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="КАЛЬКУЛЯЦИЯ" sheetId="1" r:id="Rc618bf5710ee4991"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ТЕХКАРТА" sheetId="2" r:id="Rcf6b3f3ce66e45ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="АНКЕТА" sheetId="3" r:id="R247a1d751a354304"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -758,7 +758,7 @@
         <x:f>$B$11</x:f>
         <x:v>740</x:v>
       </x:c>
-      <x:c r="C16" s="37" t="str">
+      <x:c r="C16" s="37" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="D16" s="37" t="n">
@@ -795,7 +795,7 @@
         <x:f>$B$11</x:f>
         <x:v>740</x:v>
       </x:c>
-      <x:c r="C17" s="37" t="str">
+      <x:c r="C17" s="37" t="n">
         <x:v>65</x:v>
       </x:c>
       <x:c r="D17" s="37" t="n">
@@ -2213,8 +2213,8 @@
       <x:formula1>"СОГЛАСОВАНО,ИЗМЕНИТЬ,ОТКЛОНЕНО,ТРЕБУЕТСЯ ТЕСТ,Н/П"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="date" operator="between" sqref="I5:I26">
-      <x:formula1>2026-01-01</x:formula1>
-      <x:formula2>2030-12-31</x:formula2>
+      <x:formula1>46023</x:formula1>
+      <x:formula2>47848</x:formula2>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>